<commit_message>
Update template: merge all data into single sheet
</commit_message>
<xml_diff>
--- a/global/投放效果追踪模板.xlsx
+++ b/global/投放效果追踪模板.xlsx
@@ -3,10 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="投放动作记录" sheetId="1" r:id="rId1"/>
-    <sheet name="渠道效果数据" sheetId="2" r:id="rId2"/>
-    <sheet name="转化效果数据" sheetId="3" r:id="rId3"/>
-    <sheet name="字段说明" sheetId="4" r:id="rId4"/>
+    <sheet name="投放效果追踪" sheetId="1" r:id="rId1"/>
+    <sheet name="字段说明" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -400,36 +398,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W7"/>
+  <dimension ref="A1:AL10"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" customWidth="1"/>
+    <col min="4" max="4" width="11.83203125" customWidth="1"/>
     <col min="5" max="5" width="8.83203125" customWidth="1"/>
     <col min="6" max="6" width="10.83203125" customWidth="1"/>
     <col min="7" max="7" width="12.83203125" customWidth="1"/>
     <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="50.83203125" customWidth="1"/>
-    <col min="11" max="11" width="15.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1"/>
-    <col min="13" max="13" width="10.83203125" customWidth="1"/>
-    <col min="14" max="14" width="15.83203125" customWidth="1"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1"/>
-    <col min="16" max="16" width="12.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="20.83203125" customWidth="1"/>
-    <col min="19" max="19" width="15.83203125" customWidth="1"/>
-    <col min="20" max="20" width="15.83203125" customWidth="1"/>
+    <col min="9" max="9" width="10.83203125" customWidth="1"/>
+    <col min="10" max="10" width="45.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="28.83203125" customWidth="1"/>
+    <col min="13" max="13" width="8.83203125" customWidth="1"/>
+    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="10.83203125" customWidth="1"/>
+    <col min="16" max="16" width="8.83203125" customWidth="1"/>
+    <col min="17" max="17" width="14.83203125" customWidth="1"/>
+    <col min="18" max="18" width="10.83203125" customWidth="1"/>
+    <col min="19" max="19" width="12.83203125" customWidth="1"/>
+    <col min="20" max="20" width="10.83203125" customWidth="1"/>
     <col min="21" max="21" width="12.83203125" customWidth="1"/>
-    <col min="22" max="22" width="14.83203125" customWidth="1"/>
-    <col min="23" max="23" width="10.83203125" customWidth="1"/>
+    <col min="22" max="22" width="8.83203125" customWidth="1"/>
+    <col min="23" max="23" width="9.83203125" customWidth="1"/>
+    <col min="24" max="24" width="8.83203125" customWidth="1"/>
+    <col min="25" max="25" width="8.83203125" customWidth="1"/>
+    <col min="26" max="26" width="8.83203125" customWidth="1"/>
+    <col min="27" max="27" width="9.83203125" customWidth="1"/>
+    <col min="28" max="28" width="8.83203125" customWidth="1"/>
+    <col min="29" max="29" width="8.83203125" customWidth="1"/>
+    <col min="30" max="30" width="9.83203125" customWidth="1"/>
+    <col min="31" max="31" width="10.83203125" customWidth="1"/>
+    <col min="32" max="32" width="10.83203125" customWidth="1"/>
+    <col min="33" max="33" width="11.83203125" customWidth="1"/>
+    <col min="34" max="34" width="11.83203125" customWidth="1"/>
+    <col min="35" max="35" width="11.83203125" customWidth="1"/>
+    <col min="36" max="36" width="9.83203125" customWidth="1"/>
+    <col min="37" max="37" width="8.83203125" customWidth="1"/>
+    <col min="38" max="38" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>投放效果追踪 - 投放动作记录表</v>
+        <v>投放效果追踪表 - Global &amp; SurferCloud</v>
       </c>
     </row>
     <row r="2">
@@ -439,7 +452,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>一、基础信息</v>
+        <v>【基础信息】</v>
       </c>
       <c r="B3" t="str">
         <v/>
@@ -454,7 +467,7 @@
         <v/>
       </c>
       <c r="F3" t="str">
-        <v>二、渠道信息</v>
+        <v>【渠道信息】</v>
       </c>
       <c r="G3" t="str">
         <v/>
@@ -469,7 +482,7 @@
         <v/>
       </c>
       <c r="K3" t="str">
-        <v>三、内容与定向</v>
+        <v>【内容与定向】</v>
       </c>
       <c r="L3" t="str">
         <v/>
@@ -481,10 +494,10 @@
         <v/>
       </c>
       <c r="O3" t="str">
-        <v/>
+        <v>【追踪参数】</v>
       </c>
       <c r="P3" t="str">
-        <v>四、追踪参数</v>
+        <v/>
       </c>
       <c r="Q3" t="str">
         <v/>
@@ -496,10 +509,61 @@
         <v/>
       </c>
       <c r="T3" t="str">
-        <v/>
+        <v>【成本】</v>
       </c>
       <c r="U3" t="str">
-        <v>五、成本</v>
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v>【渠道效果】</v>
+      </c>
+      <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v/>
+      </c>
+      <c r="AA3" t="str">
+        <v/>
+      </c>
+      <c r="AB3" t="str">
+        <v>【转化效果】</v>
+      </c>
+      <c r="AC3" t="str">
+        <v/>
+      </c>
+      <c r="AD3" t="str">
+        <v/>
+      </c>
+      <c r="AE3" t="str">
+        <v/>
+      </c>
+      <c r="AF3" t="str">
+        <v/>
+      </c>
+      <c r="AG3" t="str">
+        <v/>
+      </c>
+      <c r="AH3" t="str">
+        <v/>
+      </c>
+      <c r="AI3" t="str">
+        <v/>
+      </c>
+      <c r="AJ3" t="str">
+        <v>【ROI分析】</v>
+      </c>
+      <c r="AK3" t="str">
+        <v/>
+      </c>
+      <c r="AL3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -543,34 +607,79 @@
         <v>素材类型</v>
       </c>
       <c r="N4" t="str">
-        <v>目标受众</v>
+        <v>定向地区</v>
       </c>
       <c r="O4" t="str">
-        <v>定向地区</v>
+        <v>utm_source</v>
       </c>
       <c r="P4" t="str">
-        <v>utm_source</v>
+        <v>utm_medium</v>
       </c>
       <c r="Q4" t="str">
-        <v>utm_medium</v>
+        <v>utm_campaign</v>
       </c>
       <c r="R4" t="str">
-        <v>utm_campaign</v>
+        <v>utm_content</v>
       </c>
       <c r="S4" t="str">
-        <v>utm_content</v>
+        <v>自定义追踪码</v>
       </c>
       <c r="T4" t="str">
-        <v>自定义追踪码</v>
+        <v>预算(USD)</v>
       </c>
       <c r="U4" t="str">
-        <v>预算(USD)</v>
+        <v>实际花费(USD)</v>
       </c>
       <c r="V4" t="str">
-        <v>实际花费(USD)</v>
+        <v>计费方式</v>
       </c>
       <c r="W4" t="str">
-        <v>计费方式</v>
+        <v>展示量</v>
+      </c>
+      <c r="X4" t="str">
+        <v>点击量</v>
+      </c>
+      <c r="Y4" t="str">
+        <v>CTR(%)</v>
+      </c>
+      <c r="Z4" t="str">
+        <v>CPC(USD)</v>
+      </c>
+      <c r="AA4" t="str">
+        <v>CPM(USD)</v>
+      </c>
+      <c r="AB4" t="str">
+        <v>访问UV</v>
+      </c>
+      <c r="AC4" t="str">
+        <v>注册量</v>
+      </c>
+      <c r="AD4" t="str">
+        <v>注册率(%)</v>
+      </c>
+      <c r="AE4" t="str">
+        <v>实名认证数</v>
+      </c>
+      <c r="AF4" t="str">
+        <v>首充用户数</v>
+      </c>
+      <c r="AG4" t="str">
+        <v>首充金额(USD)</v>
+      </c>
+      <c r="AH4" t="str">
+        <v>累计充值(USD)</v>
+      </c>
+      <c r="AI4" t="str">
+        <v>累计消费(USD)</v>
+      </c>
+      <c r="AJ4" t="str">
+        <v>CPA(USD)</v>
+      </c>
+      <c r="AK4" t="str">
+        <v>ROI(%)</v>
+      </c>
+      <c r="AL4" t="str">
+        <v>备注</v>
       </c>
     </row>
     <row r="5">
@@ -602,46 +711,91 @@
         <v>搜索结果页</v>
       </c>
       <c r="J5" t="str">
-        <v>https://www.ucloud-global.com/en?utm_source=google&amp;utm_medium=cpc&amp;utm_campaign=cloud_hosting</v>
+        <v>https://www.ucloud-global.com/en?utm_source=google&amp;utm_medium=cpc&amp;utm_campaign=cloud_q1</v>
       </c>
       <c r="K5" t="str">
         <v>云主机推广</v>
       </c>
       <c r="L5" t="str">
-        <v>High-Performance Cloud Hosting - Start Free</v>
+        <v>High-Performance Cloud Hosting</v>
       </c>
       <c r="M5" t="str">
         <v>纯文字</v>
       </c>
       <c r="N5" t="str">
-        <v>开发者/企业</v>
+        <v>北美/欧洲</v>
       </c>
       <c r="O5" t="str">
-        <v>北美/欧洲</v>
+        <v>google</v>
       </c>
       <c r="P5" t="str">
-        <v>google</v>
+        <v>cpc</v>
       </c>
       <c r="Q5" t="str">
-        <v>cpc</v>
+        <v>cloud_q1</v>
       </c>
       <c r="R5" t="str">
-        <v>cloud_hosting_q1</v>
+        <v>text_v1</v>
       </c>
       <c r="S5" t="str">
-        <v>text_ad_v1</v>
-      </c>
-      <c r="T5" t="str">
-        <v/>
-      </c>
-      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="T5">
         <v>5000</v>
       </c>
+      <c r="U5">
+        <v>4800</v>
+      </c>
       <c r="V5" t="str">
-        <v>4800</v>
-      </c>
-      <c r="W5" t="str">
         <v>CPC</v>
+      </c>
+      <c r="W5">
+        <v>50000</v>
+      </c>
+      <c r="X5">
+        <v>1200</v>
+      </c>
+      <c r="Y5" t="str">
+        <v>=X5/W5*100</v>
+      </c>
+      <c r="Z5" t="str">
+        <v>=U5/X5</v>
+      </c>
+      <c r="AA5" t="str">
+        <v>=U5/W5*1000</v>
+      </c>
+      <c r="AB5">
+        <v>1100</v>
+      </c>
+      <c r="AC5">
+        <v>85</v>
+      </c>
+      <c r="AD5" t="str">
+        <v>=AD5/X5*100</v>
+      </c>
+      <c r="AE5">
+        <v>72</v>
+      </c>
+      <c r="AF5">
+        <v>18</v>
+      </c>
+      <c r="AG5">
+        <v>1800</v>
+      </c>
+      <c r="AH5">
+        <v>3500</v>
+      </c>
+      <c r="AI5">
+        <v>2800</v>
+      </c>
+      <c r="AJ5" t="str">
+        <v>=U5/AD5</v>
+      </c>
+      <c r="AK5" t="str">
+        <v>=(AI5-U5)/U5*100</v>
+      </c>
+      <c r="AL5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -673,46 +827,91 @@
         <v>Feed流</v>
       </c>
       <c r="J6" t="str">
-        <v>https://www.surfercloud.com/?utm_source=linkedin&amp;utm_medium=social&amp;utm_campaign=b2b_promo</v>
+        <v>https://www.surfercloud.com/?utm_source=linkedin&amp;utm_medium=social&amp;utm_campaign=b2b_feb</v>
       </c>
       <c r="K6" t="str">
         <v>B2B企业方案</v>
       </c>
       <c r="L6" t="str">
-        <v>Enterprise Cloud Solutions for Your Business</v>
+        <v>Enterprise Cloud Solutions</v>
       </c>
       <c r="M6" t="str">
         <v>图片</v>
       </c>
       <c r="N6" t="str">
-        <v>企业IT决策者</v>
+        <v>东南亚</v>
       </c>
       <c r="O6" t="str">
-        <v>东南亚</v>
+        <v>linkedin</v>
       </c>
       <c r="P6" t="str">
-        <v>linkedin</v>
+        <v>social</v>
       </c>
       <c r="Q6" t="str">
-        <v>social</v>
+        <v>b2b_feb</v>
       </c>
       <c r="R6" t="str">
-        <v>b2b_promo_feb</v>
+        <v>banner_v2</v>
       </c>
       <c r="S6" t="str">
-        <v>banner_v2</v>
-      </c>
-      <c r="T6" t="str">
         <v>ytag=B01</v>
       </c>
-      <c r="U6" t="str">
+      <c r="T6">
         <v>3000</v>
       </c>
+      <c r="U6">
+        <v>2850</v>
+      </c>
       <c r="V6" t="str">
-        <v>2850</v>
-      </c>
-      <c r="W6" t="str">
         <v>CPM</v>
+      </c>
+      <c r="W6">
+        <v>30000</v>
+      </c>
+      <c r="X6">
+        <v>450</v>
+      </c>
+      <c r="Y6" t="str">
+        <v>=X6/W6*100</v>
+      </c>
+      <c r="Z6" t="str">
+        <v>=U6/X6</v>
+      </c>
+      <c r="AA6" t="str">
+        <v>=U6/W6*1000</v>
+      </c>
+      <c r="AB6">
+        <v>420</v>
+      </c>
+      <c r="AC6">
+        <v>35</v>
+      </c>
+      <c r="AD6" t="str">
+        <v>=AD6/X6*100</v>
+      </c>
+      <c r="AE6">
+        <v>28</v>
+      </c>
+      <c r="AF6">
+        <v>8</v>
+      </c>
+      <c r="AG6">
+        <v>960</v>
+      </c>
+      <c r="AH6">
+        <v>1800</v>
+      </c>
+      <c r="AI6">
+        <v>1200</v>
+      </c>
+      <c r="AJ6" t="str">
+        <v>=U6/AD6</v>
+      </c>
+      <c r="AK6" t="str">
+        <v>=(AI6-U6)/U6*100</v>
+      </c>
+      <c r="AL6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -750,427 +949,454 @@
         <v>开发者社区推广</v>
       </c>
       <c r="L7" t="str">
-        <v>分享：海外云服务器选型经验</v>
+        <v>海外云服务器选型分享</v>
       </c>
       <c r="M7" t="str">
         <v>纯文字</v>
       </c>
       <c r="N7" t="str">
-        <v>开发者</v>
+        <v>全球华人</v>
       </c>
       <c r="O7" t="str">
-        <v>全球华人</v>
+        <v>v2ex</v>
       </c>
       <c r="P7" t="str">
-        <v>v2ex</v>
+        <v>content</v>
       </c>
       <c r="Q7" t="str">
-        <v>content</v>
+        <v>dev_community</v>
       </c>
       <c r="R7" t="str">
-        <v>dev_community</v>
+        <v>post_v1</v>
       </c>
       <c r="S7" t="str">
-        <v>post_v1</v>
-      </c>
-      <c r="T7" t="str">
-        <v/>
-      </c>
-      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="T7">
         <v>500</v>
       </c>
+      <c r="U7">
+        <v>500</v>
+      </c>
       <c r="V7" t="str">
-        <v>500</v>
-      </c>
-      <c r="W7" t="str">
         <v>固定费用</v>
+      </c>
+      <c r="W7">
+        <v>5000</v>
+      </c>
+      <c r="X7">
+        <v>320</v>
+      </c>
+      <c r="Y7" t="str">
+        <v>=X7/W7*100</v>
+      </c>
+      <c r="Z7" t="str">
+        <v>=U7/X7</v>
+      </c>
+      <c r="AA7" t="str">
+        <v>=U7/W7*1000</v>
+      </c>
+      <c r="AB7">
+        <v>300</v>
+      </c>
+      <c r="AC7">
+        <v>45</v>
+      </c>
+      <c r="AD7" t="str">
+        <v>=AD7/X7*100</v>
+      </c>
+      <c r="AE7">
+        <v>38</v>
+      </c>
+      <c r="AF7">
+        <v>12</v>
+      </c>
+      <c r="AG7">
+        <v>1500</v>
+      </c>
+      <c r="AH7">
+        <v>2200</v>
+      </c>
+      <c r="AI7">
+        <v>1800</v>
+      </c>
+      <c r="AJ7" t="str">
+        <v>=U7/AD7</v>
+      </c>
+      <c r="AK7" t="str">
+        <v>=(AI7-U7)/U7*100</v>
+      </c>
+      <c r="AL7" t="str">
+        <v>社区帖子效果好</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+      <c r="W8" t="str">
+        <v/>
+      </c>
+      <c r="X8" t="str">
+        <v/>
+      </c>
+      <c r="Y8" t="str">
+        <v/>
+      </c>
+      <c r="Z8" t="str">
+        <v/>
+      </c>
+      <c r="AA8" t="str">
+        <v/>
+      </c>
+      <c r="AB8" t="str">
+        <v/>
+      </c>
+      <c r="AC8" t="str">
+        <v/>
+      </c>
+      <c r="AD8" t="str">
+        <v/>
+      </c>
+      <c r="AE8" t="str">
+        <v/>
+      </c>
+      <c r="AF8" t="str">
+        <v/>
+      </c>
+      <c r="AG8" t="str">
+        <v/>
+      </c>
+      <c r="AH8" t="str">
+        <v/>
+      </c>
+      <c r="AI8" t="str">
+        <v/>
+      </c>
+      <c r="AJ8" t="str">
+        <v/>
+      </c>
+      <c r="AK8" t="str">
+        <v/>
+      </c>
+      <c r="AL8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+      <c r="W9" t="str">
+        <v/>
+      </c>
+      <c r="X9" t="str">
+        <v/>
+      </c>
+      <c r="Y9" t="str">
+        <v/>
+      </c>
+      <c r="Z9" t="str">
+        <v/>
+      </c>
+      <c r="AA9" t="str">
+        <v/>
+      </c>
+      <c r="AB9" t="str">
+        <v/>
+      </c>
+      <c r="AC9" t="str">
+        <v/>
+      </c>
+      <c r="AD9" t="str">
+        <v/>
+      </c>
+      <c r="AE9" t="str">
+        <v/>
+      </c>
+      <c r="AF9" t="str">
+        <v/>
+      </c>
+      <c r="AG9" t="str">
+        <v/>
+      </c>
+      <c r="AH9" t="str">
+        <v/>
+      </c>
+      <c r="AI9" t="str">
+        <v/>
+      </c>
+      <c r="AJ9" t="str">
+        <v/>
+      </c>
+      <c r="AK9" t="str">
+        <v/>
+      </c>
+      <c r="AL9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v/>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str">
+        <v/>
+      </c>
+      <c r="V10" t="str">
+        <v/>
+      </c>
+      <c r="W10" t="str">
+        <v/>
+      </c>
+      <c r="X10" t="str">
+        <v/>
+      </c>
+      <c r="Y10" t="str">
+        <v/>
+      </c>
+      <c r="Z10" t="str">
+        <v/>
+      </c>
+      <c r="AA10" t="str">
+        <v/>
+      </c>
+      <c r="AB10" t="str">
+        <v/>
+      </c>
+      <c r="AC10" t="str">
+        <v/>
+      </c>
+      <c r="AD10" t="str">
+        <v/>
+      </c>
+      <c r="AE10" t="str">
+        <v/>
+      </c>
+      <c r="AF10" t="str">
+        <v/>
+      </c>
+      <c r="AG10" t="str">
+        <v/>
+      </c>
+      <c r="AH10" t="str">
+        <v/>
+      </c>
+      <c r="AI10" t="str">
+        <v/>
+      </c>
+      <c r="AJ10" t="str">
+        <v/>
+      </c>
+      <c r="AK10" t="str">
+        <v/>
+      </c>
+      <c r="AL10" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:W1"/>
+    <mergeCell ref="A1:AL1"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AL10"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:E48"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
-    <col min="8" max="8" width="30.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>渠道效果数据（渠道后台数据）</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>投放ID</v>
-      </c>
-      <c r="B3" t="str">
-        <v>统计日期</v>
-      </c>
-      <c r="C3" t="str">
-        <v>展示量</v>
-      </c>
-      <c r="D3" t="str">
-        <v>点击量</v>
-      </c>
-      <c r="E3" t="str">
-        <v>CTR(%)</v>
-      </c>
-      <c r="F3" t="str">
-        <v>CPC(USD)</v>
-      </c>
-      <c r="G3" t="str">
-        <v>CPM(USD)</v>
-      </c>
-      <c r="H3" t="str">
-        <v>备注</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>ADV-2026-001</v>
-      </c>
-      <c r="B4" t="str">
-        <v>2026-01-15</v>
-      </c>
-      <c r="C4" t="str">
-        <v>50000</v>
-      </c>
-      <c r="D4" t="str">
-        <v>1200</v>
-      </c>
-      <c r="E4" t="str">
-        <v>2.4%</v>
-      </c>
-      <c r="F4" t="str">
-        <v>4.00</v>
-      </c>
-      <c r="G4" t="str">
-        <v>96</v>
-      </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>ADV-2026-001</v>
-      </c>
-      <c r="B5" t="str">
-        <v>2026-01-16</v>
-      </c>
-      <c r="C5" t="str">
-        <v>48000</v>
-      </c>
-      <c r="D5" t="str">
-        <v>1150</v>
-      </c>
-      <c r="E5" t="str">
-        <v>2.4%</v>
-      </c>
-      <c r="F5" t="str">
-        <v>4.17</v>
-      </c>
-      <c r="G5" t="str">
-        <v>100</v>
-      </c>
-      <c r="H5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>ADV-2026-002</v>
-      </c>
-      <c r="B6" t="str">
-        <v>2026-02-01</v>
-      </c>
-      <c r="C6" t="str">
-        <v>30000</v>
-      </c>
-      <c r="D6" t="str">
-        <v>450</v>
-      </c>
-      <c r="E6" t="str">
-        <v>1.5%</v>
-      </c>
-      <c r="F6" t="str">
-        <v>6.33</v>
-      </c>
-      <c r="G6" t="str">
-        <v>95</v>
-      </c>
-      <c r="H6" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>ADV-2026-003</v>
-      </c>
-      <c r="B7" t="str">
-        <v>2026-02-10</v>
-      </c>
-      <c r="C7" t="str">
-        <v>5000</v>
-      </c>
-      <c r="D7" t="str">
-        <v>320</v>
-      </c>
-      <c r="E7" t="str">
-        <v>6.4%</v>
-      </c>
-      <c r="F7" t="str">
-        <v>1.56</v>
-      </c>
-      <c r="G7" t="str">
-        <v>100</v>
-      </c>
-      <c r="H7" t="str">
-        <v>社区帖子热度高</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
-  </mergeCells>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
-  <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" customWidth="1"/>
-    <col min="12" max="12" width="10.83203125" customWidth="1"/>
-    <col min="13" max="13" width="10.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>转化效果数据（站点后台数据）</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>投放ID</v>
-      </c>
-      <c r="B3" t="str">
-        <v>统计周期</v>
-      </c>
-      <c r="C3" t="str">
-        <v>访问UV</v>
-      </c>
-      <c r="D3" t="str">
-        <v>注册量</v>
-      </c>
-      <c r="E3" t="str">
-        <v>注册率(%)</v>
-      </c>
-      <c r="F3" t="str">
-        <v>实名认证数</v>
-      </c>
-      <c r="G3" t="str">
-        <v>首充用户数</v>
-      </c>
-      <c r="H3" t="str">
-        <v>首充金额(USD)</v>
-      </c>
-      <c r="I3" t="str">
-        <v>付费率(%)</v>
-      </c>
-      <c r="J3" t="str">
-        <v>累计充值(USD)</v>
-      </c>
-      <c r="K3" t="str">
-        <v>累计消费(USD)</v>
-      </c>
-      <c r="L3" t="str">
-        <v>CPA(USD)</v>
-      </c>
-      <c r="M3" t="str">
-        <v>ROI(%)</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>ADV-2026-001</v>
-      </c>
-      <c r="B4" t="str">
-        <v>2026-01全月</v>
-      </c>
-      <c r="C4" t="str">
-        <v>1100</v>
-      </c>
-      <c r="D4" t="str">
-        <v>85</v>
-      </c>
-      <c r="E4" t="str">
-        <v>7.7%</v>
-      </c>
-      <c r="F4" t="str">
-        <v>72</v>
-      </c>
-      <c r="G4" t="str">
-        <v>18</v>
-      </c>
-      <c r="H4" t="str">
-        <v>1800</v>
-      </c>
-      <c r="I4" t="str">
-        <v>21.2%</v>
-      </c>
-      <c r="J4" t="str">
-        <v>3500</v>
-      </c>
-      <c r="K4" t="str">
-        <v>2800</v>
-      </c>
-      <c r="L4" t="str">
-        <v>56.47</v>
-      </c>
-      <c r="M4" t="str">
-        <v>-27%</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>ADV-2026-002</v>
-      </c>
-      <c r="B5" t="str">
-        <v>2026-02全月</v>
-      </c>
-      <c r="C5" t="str">
-        <v>420</v>
-      </c>
-      <c r="D5" t="str">
-        <v>35</v>
-      </c>
-      <c r="E5" t="str">
-        <v>8.3%</v>
-      </c>
-      <c r="F5" t="str">
-        <v>28</v>
-      </c>
-      <c r="G5" t="str">
-        <v>8</v>
-      </c>
-      <c r="H5" t="str">
-        <v>960</v>
-      </c>
-      <c r="I5" t="str">
-        <v>22.9%</v>
-      </c>
-      <c r="J5" t="str">
-        <v>1800</v>
-      </c>
-      <c r="K5" t="str">
-        <v>1200</v>
-      </c>
-      <c r="L5" t="str">
-        <v>81.43</v>
-      </c>
-      <c r="M5" t="str">
-        <v>-37%</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>ADV-2026-003</v>
-      </c>
-      <c r="B6" t="str">
-        <v>2026-02-10~20</v>
-      </c>
-      <c r="C6" t="str">
-        <v>300</v>
-      </c>
-      <c r="D6" t="str">
-        <v>45</v>
-      </c>
-      <c r="E6" t="str">
-        <v>15.0%</v>
-      </c>
-      <c r="F6" t="str">
-        <v>38</v>
-      </c>
-      <c r="G6" t="str">
-        <v>12</v>
-      </c>
-      <c r="H6" t="str">
-        <v>1500</v>
-      </c>
-      <c r="I6" t="str">
-        <v>26.7%</v>
-      </c>
-      <c r="J6" t="str">
-        <v>2200</v>
-      </c>
-      <c r="K6" t="str">
-        <v>1800</v>
-      </c>
-      <c r="L6" t="str">
-        <v>11.11</v>
-      </c>
-      <c r="M6" t="str">
-        <v>260%</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:M1"/>
-  </mergeCells>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D38"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="50.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="25.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1185,7 +1411,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>类别</v>
+        <v>分组</v>
       </c>
       <c r="B3" t="str">
         <v>字段名</v>
@@ -1194,6 +1420,9 @@
         <v>说明</v>
       </c>
       <c r="D3" t="str">
+        <v>填写来源</v>
+      </c>
+      <c r="E3" t="str">
         <v>示例值</v>
       </c>
     </row>
@@ -1205,9 +1434,12 @@
         <v>投放ID</v>
       </c>
       <c r="C4" t="str">
-        <v>唯一标识符，建议格式：ADV-年份-序号</v>
+        <v>唯一标识符</v>
       </c>
       <c r="D4" t="str">
+        <v>自定义</v>
+      </c>
+      <c r="E4" t="str">
         <v>ADV-2026-001</v>
       </c>
     </row>
@@ -1222,6 +1454,9 @@
         <v>Global 或 SurferCloud</v>
       </c>
       <c r="D5" t="str">
+        <v>选择</v>
+      </c>
+      <c r="E5" t="str">
         <v>Global</v>
       </c>
     </row>
@@ -1236,6 +1471,9 @@
         <v>投放开始日期</v>
       </c>
       <c r="D6" t="str">
+        <v>填写</v>
+      </c>
+      <c r="E6" t="str">
         <v>2026-01-15</v>
       </c>
     </row>
@@ -1247,9 +1485,12 @@
         <v>结束日期</v>
       </c>
       <c r="C7" t="str">
-        <v>投放结束日期，持续中可留空</v>
+        <v>投放结束日期</v>
       </c>
       <c r="D7" t="str">
+        <v>填写</v>
+      </c>
+      <c r="E7" t="str">
         <v>2026-01-31</v>
       </c>
     </row>
@@ -1261,9 +1502,12 @@
         <v>负责人</v>
       </c>
       <c r="C8" t="str">
-        <v>执行投放的同事姓名</v>
+        <v>执行投放的同事</v>
       </c>
       <c r="D8" t="str">
+        <v>填写</v>
+      </c>
+      <c r="E8" t="str">
         <v>张三</v>
       </c>
     </row>
@@ -1278,6 +1522,9 @@
         <v/>
       </c>
       <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
         <v/>
       </c>
     </row>
@@ -1292,6 +1539,9 @@
         <v>搜索引擎/社交媒体/内容平台/联盟广告/其他</v>
       </c>
       <c r="D10" t="str">
+        <v>选择</v>
+      </c>
+      <c r="E10" t="str">
         <v>搜索引擎</v>
       </c>
     </row>
@@ -1303,9 +1553,12 @@
         <v>渠道平台</v>
       </c>
       <c r="C11" t="str">
-        <v>Google Ads/Facebook/LinkedIn/Twitter/Reddit/知乎/V2EX等</v>
+        <v>Google/Facebook/LinkedIn/V2EX等</v>
       </c>
       <c r="D11" t="str">
+        <v>填写</v>
+      </c>
+      <c r="E11" t="str">
         <v>Google Ads</v>
       </c>
     </row>
@@ -1317,9 +1570,12 @@
         <v>投放形式</v>
       </c>
       <c r="C12" t="str">
-        <v>SEM搜索/展示广告/信息流/视频广告/KOL合作/软文</v>
+        <v>SEM/展示广告/信息流/视频/软文等</v>
       </c>
       <c r="D12" t="str">
+        <v>选择</v>
+      </c>
+      <c r="E12" t="str">
         <v>SEM搜索</v>
       </c>
     </row>
@@ -1334,6 +1590,9 @@
         <v>具体展示位置</v>
       </c>
       <c r="D13" t="str">
+        <v>填写</v>
+      </c>
+      <c r="E13" t="str">
         <v>搜索结果页</v>
       </c>
     </row>
@@ -1345,9 +1604,12 @@
         <v>落地页URL</v>
       </c>
       <c r="C14" t="str">
-        <v>用户点击后到达的页面，需包含UTM参数</v>
+        <v>包含UTM参数的完整URL</v>
       </c>
       <c r="D14" t="str">
+        <v>填写</v>
+      </c>
+      <c r="E14" t="str">
         <v>https://...?utm_xxx</v>
       </c>
     </row>
@@ -1362,6 +1624,9 @@
         <v/>
       </c>
       <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
         <v/>
       </c>
     </row>
@@ -1376,7 +1641,10 @@
         <v>投放主题/卖点</v>
       </c>
       <c r="D16" t="str">
-        <v>新用户免费试用</v>
+        <v>填写</v>
+      </c>
+      <c r="E16" t="str">
+        <v>云主机推广</v>
       </c>
     </row>
     <row r="17">
@@ -1390,6 +1658,9 @@
         <v>核心文案内容</v>
       </c>
       <c r="D17" t="str">
+        <v>填写</v>
+      </c>
+      <c r="E17" t="str">
         <v>Free $100 Credit</v>
       </c>
     </row>
@@ -1401,9 +1672,12 @@
         <v>素材类型</v>
       </c>
       <c r="C18" t="str">
-        <v>图片/视频/纯文字/轮播图</v>
+        <v>图片/视频/纯文字</v>
       </c>
       <c r="D18" t="str">
+        <v>选择</v>
+      </c>
+      <c r="E18" t="str">
         <v>图片</v>
       </c>
     </row>
@@ -1412,41 +1686,50 @@
         <v>内容定向</v>
       </c>
       <c r="B19" t="str">
-        <v>目标受众</v>
+        <v>定向地区</v>
       </c>
       <c r="C19" t="str">
-        <v>定向人群描述</v>
+        <v>投放地域</v>
       </c>
       <c r="D19" t="str">
-        <v>开发者/企业用户</v>
+        <v>填写</v>
+      </c>
+      <c r="E19" t="str">
+        <v>北美/欧洲</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>内容定向</v>
+        <v/>
       </c>
       <c r="B20" t="str">
-        <v>定向地区</v>
+        <v/>
       </c>
       <c r="C20" t="str">
-        <v>投放地域</v>
+        <v/>
       </c>
       <c r="D20" t="str">
-        <v>北美/欧洲/东南亚/全球</v>
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v/>
+        <v>追踪参数</v>
       </c>
       <c r="B21" t="str">
-        <v/>
+        <v>utm_source</v>
       </c>
       <c r="C21" t="str">
-        <v/>
+        <v>流量来源</v>
       </c>
       <c r="D21" t="str">
-        <v/>
+        <v>填写</v>
+      </c>
+      <c r="E21" t="str">
+        <v>google</v>
       </c>
     </row>
     <row r="22">
@@ -1454,13 +1737,16 @@
         <v>追踪参数</v>
       </c>
       <c r="B22" t="str">
-        <v>utm_source</v>
+        <v>utm_medium</v>
       </c>
       <c r="C22" t="str">
-        <v>流量来源</v>
+        <v>媒介类型</v>
       </c>
       <c r="D22" t="str">
-        <v>google/facebook/linkedin</v>
+        <v>填写</v>
+      </c>
+      <c r="E22" t="str">
+        <v>cpc</v>
       </c>
     </row>
     <row r="23">
@@ -1468,13 +1754,16 @@
         <v>追踪参数</v>
       </c>
       <c r="B23" t="str">
-        <v>utm_medium</v>
+        <v>utm_campaign</v>
       </c>
       <c r="C23" t="str">
-        <v>媒介类型</v>
+        <v>活动名称</v>
       </c>
       <c r="D23" t="str">
-        <v>cpc/cpm/social/email</v>
+        <v>填写</v>
+      </c>
+      <c r="E23" t="str">
+        <v>cloud_q1</v>
       </c>
     </row>
     <row r="24">
@@ -1482,13 +1771,16 @@
         <v>追踪参数</v>
       </c>
       <c r="B24" t="str">
-        <v>utm_campaign</v>
+        <v>utm_content</v>
       </c>
       <c r="C24" t="str">
-        <v>活动名称</v>
+        <v>素材版本</v>
       </c>
       <c r="D24" t="str">
-        <v>spring_promo_2026</v>
+        <v>填写</v>
+      </c>
+      <c r="E24" t="str">
+        <v>text_v1</v>
       </c>
     </row>
     <row r="25">
@@ -1496,41 +1788,50 @@
         <v>追踪参数</v>
       </c>
       <c r="B25" t="str">
-        <v>utm_content</v>
+        <v>自定义追踪码</v>
       </c>
       <c r="C25" t="str">
-        <v>区分素材版本</v>
+        <v>内部标识如ytag</v>
       </c>
       <c r="D25" t="str">
-        <v>banner_v1</v>
+        <v>填写</v>
+      </c>
+      <c r="E25" t="str">
+        <v>ytag=A03</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>追踪参数</v>
+        <v/>
       </c>
       <c r="B26" t="str">
-        <v>自定义追踪码</v>
+        <v/>
       </c>
       <c r="C26" t="str">
-        <v>内部追踪标识（如ytag）</v>
+        <v/>
       </c>
       <c r="D26" t="str">
-        <v>ytag=A03</v>
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v/>
+        <v>成本</v>
       </c>
       <c r="B27" t="str">
-        <v/>
+        <v>预算(USD)</v>
       </c>
       <c r="C27" t="str">
-        <v/>
+        <v>计划投入金额</v>
       </c>
       <c r="D27" t="str">
-        <v/>
+        <v>填写</v>
+      </c>
+      <c r="E27" t="str">
+        <v>5000</v>
       </c>
     </row>
     <row r="28">
@@ -1538,13 +1839,16 @@
         <v>成本</v>
       </c>
       <c r="B28" t="str">
-        <v>预算(USD)</v>
+        <v>实际花费(USD)</v>
       </c>
       <c r="C28" t="str">
-        <v>计划投入金额</v>
+        <v>实际消耗金额</v>
       </c>
       <c r="D28" t="str">
-        <v>5000</v>
+        <v>渠道后台</v>
+      </c>
+      <c r="E28" t="str">
+        <v>4800</v>
       </c>
     </row>
     <row r="29">
@@ -1552,147 +1856,347 @@
         <v>成本</v>
       </c>
       <c r="B29" t="str">
-        <v>实际花费(USD)</v>
+        <v>计费方式</v>
       </c>
       <c r="C29" t="str">
-        <v>实际消耗金额</v>
+        <v>CPC/CPM/CPA/固定费用</v>
       </c>
       <c r="D29" t="str">
-        <v>4800</v>
+        <v>选择</v>
+      </c>
+      <c r="E29" t="str">
+        <v>CPC</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>成本</v>
+        <v/>
       </c>
       <c r="B30" t="str">
-        <v>计费方式</v>
+        <v/>
       </c>
       <c r="C30" t="str">
-        <v>CPC/CPM/CPA/固定费用</v>
+        <v/>
       </c>
       <c r="D30" t="str">
-        <v>CPC</v>
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v/>
+        <v>渠道效果</v>
       </c>
       <c r="B31" t="str">
-        <v/>
+        <v>展示量</v>
       </c>
       <c r="C31" t="str">
-        <v/>
+        <v>广告展示次数</v>
       </c>
       <c r="D31" t="str">
-        <v/>
+        <v>渠道后台</v>
+      </c>
+      <c r="E31" t="str">
+        <v>50000</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>效果指标</v>
+        <v>渠道效果</v>
       </c>
       <c r="B32" t="str">
-        <v>展示量</v>
+        <v>点击量</v>
       </c>
       <c r="C32" t="str">
-        <v>广告展示次数（渠道后台）</v>
+        <v>广告点击次数</v>
       </c>
       <c r="D32" t="str">
-        <v>50000</v>
+        <v>渠道后台</v>
+      </c>
+      <c r="E32" t="str">
+        <v>1200</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>效果指标</v>
+        <v>渠道效果</v>
       </c>
       <c r="B33" t="str">
-        <v>点击量</v>
+        <v>CTR(%)</v>
       </c>
       <c r="C33" t="str">
-        <v>广告点击次数（渠道后台）</v>
+        <v>点击率（自动计算）</v>
       </c>
       <c r="D33" t="str">
-        <v>1200</v>
+        <v>公式</v>
+      </c>
+      <c r="E33" t="str">
+        <v>=点击/展示*100</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>效果指标</v>
+        <v>渠道效果</v>
       </c>
       <c r="B34" t="str">
-        <v>CTR</v>
+        <v>CPC(USD)</v>
       </c>
       <c r="C34" t="str">
-        <v>点击率 = 点击/展示</v>
+        <v>单次点击成本（自动计算）</v>
       </c>
       <c r="D34" t="str">
-        <v>2.4%</v>
+        <v>公式</v>
+      </c>
+      <c r="E34" t="str">
+        <v>=花费/点击</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>效果指标</v>
+        <v>渠道效果</v>
       </c>
       <c r="B35" t="str">
-        <v>注册量</v>
+        <v>CPM(USD)</v>
       </c>
       <c r="C35" t="str">
-        <v>新用户注册数（站点后台）</v>
+        <v>千次展示成本（自动计算）</v>
       </c>
       <c r="D35" t="str">
-        <v>85</v>
+        <v>公式</v>
+      </c>
+      <c r="E35" t="str">
+        <v>=花费/展示*1000</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>效果指标</v>
+        <v/>
       </c>
       <c r="B36" t="str">
-        <v>首充用户数</v>
+        <v/>
       </c>
       <c r="C36" t="str">
-        <v>首次付费用户数</v>
+        <v/>
       </c>
       <c r="D36" t="str">
-        <v>18</v>
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>效果指标</v>
+        <v>转化效果</v>
       </c>
       <c r="B37" t="str">
-        <v>CPA</v>
+        <v>访问UV</v>
       </c>
       <c r="C37" t="str">
-        <v>单注册成本 = 花费/注册量</v>
+        <v>独立访客数</v>
       </c>
       <c r="D37" t="str">
-        <v>$56.47</v>
+        <v>站点统计</v>
+      </c>
+      <c r="E37" t="str">
+        <v>1100</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>效果指标</v>
+        <v>转化效果</v>
       </c>
       <c r="B38" t="str">
-        <v>ROI</v>
+        <v>注册量</v>
       </c>
       <c r="C38" t="str">
-        <v>投资回报率 = (收入-成本)/成本</v>
+        <v>新用户注册数</v>
       </c>
       <c r="D38" t="str">
-        <v>150%</v>
+        <v>后台数据</v>
+      </c>
+      <c r="E38" t="str">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>转化效果</v>
+      </c>
+      <c r="B39" t="str">
+        <v>注册率(%)</v>
+      </c>
+      <c r="C39" t="str">
+        <v>注册转化率（自动计算）</v>
+      </c>
+      <c r="D39" t="str">
+        <v>公式</v>
+      </c>
+      <c r="E39" t="str">
+        <v>=注册/点击*100</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>转化效果</v>
+      </c>
+      <c r="B40" t="str">
+        <v>实名认证数</v>
+      </c>
+      <c r="C40" t="str">
+        <v>完成实名的用户</v>
+      </c>
+      <c r="D40" t="str">
+        <v>后台数据</v>
+      </c>
+      <c r="E40" t="str">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>转化效果</v>
+      </c>
+      <c r="B41" t="str">
+        <v>首充用户数</v>
+      </c>
+      <c r="C41" t="str">
+        <v>首次付费用户数</v>
+      </c>
+      <c r="D41" t="str">
+        <v>后台数据</v>
+      </c>
+      <c r="E41" t="str">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>转化效果</v>
+      </c>
+      <c r="B42" t="str">
+        <v>首充金额(USD)</v>
+      </c>
+      <c r="C42" t="str">
+        <v>首次充值总金额</v>
+      </c>
+      <c r="D42" t="str">
+        <v>后台数据</v>
+      </c>
+      <c r="E42" t="str">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>转化效果</v>
+      </c>
+      <c r="B43" t="str">
+        <v>累计充值(USD)</v>
+      </c>
+      <c r="C43" t="str">
+        <v>用户累计充值</v>
+      </c>
+      <c r="D43" t="str">
+        <v>后台数据</v>
+      </c>
+      <c r="E43" t="str">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>转化效果</v>
+      </c>
+      <c r="B44" t="str">
+        <v>累计消费(USD)</v>
+      </c>
+      <c r="C44" t="str">
+        <v>用户实际消费</v>
+      </c>
+      <c r="D44" t="str">
+        <v>后台数据</v>
+      </c>
+      <c r="E44" t="str">
+        <v>2800</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v/>
+      </c>
+      <c r="B45" t="str">
+        <v/>
+      </c>
+      <c r="C45" t="str">
+        <v/>
+      </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>ROI分析</v>
+      </c>
+      <c r="B46" t="str">
+        <v>CPA(USD)</v>
+      </c>
+      <c r="C46" t="str">
+        <v>单注册成本（自动计算）</v>
+      </c>
+      <c r="D46" t="str">
+        <v>公式</v>
+      </c>
+      <c r="E46" t="str">
+        <v>=花费/注册量</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>ROI分析</v>
+      </c>
+      <c r="B47" t="str">
+        <v>ROI(%)</v>
+      </c>
+      <c r="C47" t="str">
+        <v>投资回报率（自动计算）</v>
+      </c>
+      <c r="D47" t="str">
+        <v>公式</v>
+      </c>
+      <c r="E47" t="str">
+        <v>=(消费-花费)/花费*100</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>ROI分析</v>
+      </c>
+      <c r="B48" t="str">
+        <v>备注</v>
+      </c>
+      <c r="C48" t="str">
+        <v>补充说明</v>
+      </c>
+      <c r="D48" t="str">
+        <v>填写</v>
+      </c>
+      <c r="E48" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E48"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>